<commit_message>
Add audit dashboard and refresh workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZRcoyLH9Dpj4dpsaCuSfy
</commit_message>
<xml_diff>
--- a/reports/2026-10-01-audit.xlsx
+++ b/reports/2026-10-01-audit.xlsx
@@ -1385,7 +1385,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Same amount as 9/15 bill, 8/26 tag</t>
+          <t>Same amount as 9/15 bill, 8/26 tag (not counted in $ at risk)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1398,9 +1398,7 @@
           <t>569-479-000 8/26</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>275.32</v>
-      </c>
+      <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>9/9</t>
@@ -1451,7 +1449,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>August bill</t>
+          <t>August bill (not counted in $ at risk)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1464,9 +1462,7 @@
           <t>569-479-000 8/26</t>
         </is>
       </c>
-      <c r="H10" s="4" t="n">
-        <v>385.81</v>
-      </c>
+      <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>8/17</t>
@@ -1517,7 +1513,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Second Sept bill</t>
+          <t>Second Sept bill (not counted in $ at risk)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1530,9 +1526,7 @@
           <t>569-479-000 9/26</t>
         </is>
       </c>
-      <c r="H11" s="4" t="n">
-        <v>144.87</v>
-      </c>
+      <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>9/28</t>

</xml_diff>

<commit_message>
Dashboard: clearer completeness banner; drop email row from gaps
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZRcoyLH9Dpj4dpsaCuSfy
</commit_message>
<xml_diff>
--- a/reports/2026-10-01-audit.xlsx
+++ b/reports/2026-10-01-audit.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Data tie-out" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gaps'!$A$1:$E$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gaps'!$A$1:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$N$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Open items'!$A$1:$C$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Markup pairs'!$A$1:$I$85</definedName>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Gmail connector has no read/send permission (Insufficient scope).</t>
+          <t>Gmail has no read permission (Insufficient scope), so AppFolio report emails could not be checked.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -532,22 +532,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Report email</t>
+          <t>Audit rule files</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NOT SENT</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Same Gmail permission error.</t>
+          <t>Repo was empty (no CLAUDE.md, no audit/ files, no prior reports). Used rules you pasted.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Reconnect Gmail; email text is ready.</t>
+          <t>Commit the rules + OPEN_ITEMS to the repo so daily runs are consistent.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -559,49 +559,49 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Audit rule files</t>
+          <t>'New since yesterday' &amp; days-open</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>CAN'T COMPUTE</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Repo was empty (no CLAUDE.md, no audit/ files, no prior reports). Used rules you pasted.</t>
+          <t>No prior report; open items have no open dates.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Commit the rules + OPEN_ITEMS to the repo so daily runs are consistent.</t>
+          <t>Add open dates to OPEN_ITEMS; today's report becomes the baseline.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>'New since yesterday' &amp; days-open</t>
+          <t>Check 2: effective fee rate vs setting</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CAN'T COMPUTE</t>
+          <t>NOT RUN</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>No prior report; open items have no open dates.</t>
+          <t>Rent collected / fee charges by property not pulled.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Add open dates to OPEN_ITEMS; today's report becomes the baseline.</t>
+          <t>Needs a rent-collected report per property joined to Management Fee lines.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Check 2: effective fee rate vs setting</t>
+          <t>Check 3: bill on inactive property / past contract end</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -623,12 +623,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Rent collected / fee charges by property not pulled.</t>
+          <t>Property status &amp; contract dates not pulled for all properties.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Needs a rent-collected report per property joined to Management Fee lines.</t>
+          <t>Pull property report with status + contract end; join to bill lines.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -640,7 +640,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Check 3: bill on inactive property / past contract end</t>
+          <t>Check 3: vendor billing a property first time this year &gt;$500</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Property status &amp; contract dates not pulled for all properties.</t>
+          <t>Vendor is not a column in expense-distribution; needs get_bill per bill.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Pull property report with status + contract end; join to bill lines.</t>
+          <t>Pull list_bills with payee and join by reference.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -667,22 +667,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Check 3: vendor billing a property first time this year &gt;$500</t>
+          <t>Check 5a: resident-pays utilities</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Vendor is not a column in expense-distribution; needs get_bill per bill.</t>
+          <t>Only lines whose description/reference names the utility could be classified; many later-month utility lines have blank descriptions.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Pull list_bills with payee and join by reference.</t>
+          <t>Open bills with get_bill / pull payee to classify the rest.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -694,7 +694,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Check 5a: resident-pays utilities</t>
+          <t>Check 5b: leaks/spikes</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -704,12 +704,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Only lines whose description/reference names the utility could be classified; many later-month utility lines have blank descriptions.</t>
+          <t>Only trailing-3-month baseline (no 2025 data pulled); only 22 accounts with water/sewer wording and 3 months history tested.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Open bills with get_bill / pull payee to classify the rest.</t>
+          <t>Pull 2025 bills; classify accounts by payee (City of / Water District).</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Check 5b: leaks/spikes</t>
+          <t>Blank 'Property Code' lines</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -731,12 +731,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Only trailing-3-month baseline (no 2025 data pulled); only 22 accounts with water/sewer wording and 3 months history tested.</t>
+          <t>6 opened with get_bill; blank code is not always 'no property' (e.g. bills 27012, 27157 are on 5415 W Minton Ave). See sheet 'Blank property lines'.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Pull 2025 bills; classify accounts by payee (City of / Water District).</t>
+          <t>Open each listed bill and confirm the property/owner.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -748,7 +748,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Blank 'Property Code' lines</t>
+          <t>Same-building different-rate check (Rentvine)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -758,39 +758,39 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>6 opened with get_bill; blank code is not always 'no property' (e.g. bills 27012, 27157 are on 5415 W Minton Ave). See sheet 'Blank property lines'.</t>
+          <t>Only checked properties on non-standard settings + AppFolio owner view.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Open each listed bill and confirm the property/owner.</t>
+          <t>Compare rates by owner across all 423 active Rentvine properties.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Same-building different-rate check (Rentvine)</t>
+          <t>Unit management fee report</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>SKIPPED (known)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Only checked properties on non-standard settings + AppFolio owner view.</t>
+          <t>Fee income account not set in accounting settings.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Compare rates by owner across all 423 active Rentvine properties.</t>
+          <t>Set fee income account in Rentvine accounting settings.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -802,59 +802,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Unit management fee report</t>
+          <t>Month pull method</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SKIPPED (known)</t>
+          <t>NOTE</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Fee income account not set in accounting settings.</t>
+          <t>Pulled full monthly CSV exports instead of 150-row pages; row counts and $ totals matched headers for all 10 months (40,596 rows).</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Set fee income account in Rentvine accounting settings.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Month pull method</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Pulled full monthly CSV exports instead of 150-row pages; row counts and $ totals matched headers for all 10 months (40,596 rows).</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>None.</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
           <t>Info</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E14"/>
+  <autoFilter ref="A1:E13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correct AppFolio status (bills not audited, Gmail not needed); solid underlines
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZRcoyLH9Dpj4dpsaCuSfy
</commit_message>
<xml_diff>
--- a/reports/2026-10-01-audit.xlsx
+++ b/reports/2026-10-01-audit.xlsx
@@ -505,22 +505,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AppFolio Phase 2 (report emails)</t>
+          <t>AppFolio bills and renewals</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>NOT AUDITED</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Gmail has no read permission (Insufficient scope), so AppFolio report emails could not be checked.</t>
+          <t>Only AppFolio fee settings were checked. The pasted instructions said AppFolio could not return bills, but AppFolio is connected and does (tested today: 143 bills in the last 7 days). I did not run the bill checks on it. Gmail is not needed for this.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Reconnect Gmail with read+send scope, then rerun.</t>
+          <t>Run Checks 1, 3, 4, 5 against AppFolio bills (month by month, like Rentvine).</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">

</xml_diff>